<commit_message>
Auto commit 17-07-2025 12:30:51.93
</commit_message>
<xml_diff>
--- a/Templates/Compressor Pump Installation.xlsx
+++ b/Templates/Compressor Pump Installation.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20325"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Core i5 GAMING\Desktop\estimate-drafter\Templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{6BB56358-9C56-4AF0-A536-23B85935C128}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19425" windowHeight="11025" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19420" windowHeight="11020"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Flushing (Developing) Borewell (Code: GWDDR105)</t>
   </si>
@@ -31,9 +25,6 @@
     <t>Compressor pump fitting charge (Code: GWDDR055)</t>
   </si>
   <si>
-    <t>Providing and fixing G.I. pipes complete with G.I fittings including trenching and refilling etc. External work 25 mm dia nominal bore (18.12.3) (Code: GWDDR243)</t>
-  </si>
-  <si>
     <t>20 mm dia HDPE pipe (DG) (8kg) (Code: GWDMR076)</t>
   </si>
   <si>
@@ -67,29 +58,19 @@
     <t>Installation of Single Phase Panel board where new electricity connection is required (Excluding Motor Starter) (Code: GWDDR363)</t>
   </si>
   <si>
-    <t>GI Bend 40 mm (Code: GWDMR053)</t>
-  </si>
-  <si>
-    <t>GI Socket 40 mm (Code: GWDMR057)</t>
+    <t>Providing and fixing G.I. pipes complete with G.I fittings: 15 mm dia nominal bore (Code: GWDDR377)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -134,25 +115,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,22 +435,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="56.5703125" style="4" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="56.54296875" style="4" customWidth="1"/>
+    <col min="2" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -483,7 +458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -491,7 +466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -499,115 +474,99 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="60" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="72.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="75" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" ht="58" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit 17-07-2025 13:24:50.54
</commit_message>
<xml_diff>
--- a/Templates/Compressor Pump Installation.xlsx
+++ b/Templates/Compressor Pump Installation.xlsx
@@ -52,13 +52,13 @@
     <t>Metallic Pump House of size 1.2 x 0.9 x 2 m (Code: GWDDR006)</t>
   </si>
   <si>
-    <t>S &amp; F Motor starters of the following ratings Submersible pump controllers with ammeter,DPMCB for single phase 2 HP submersible motor pumps (DOL) (90.14.28.13) (Code: GWDDR134)</t>
-  </si>
-  <si>
     <t>Installation of Single Phase Panel board where new electricity connection is required (Excluding Motor Starter) (Code: GWDDR363)</t>
   </si>
   <si>
     <t>Providing and fixing G.I. pipes complete with G.I fittings: 15 mm dia nominal bore (Code: GWDDR377)</t>
+  </si>
+  <si>
+    <t>S &amp; F Single phase starters suitable for Compressor pump upto 2HP (Code: GWDDR368)</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -476,7 +476,7 @@
     </row>
     <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2">
         <v>15</v>
@@ -556,15 +556,15 @@
     </row>
     <row r="14" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="58" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="29" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2">
         <v>1</v>

</xml_diff>